<commit_message>
fix: ItemEffectTable.csv를 .cs에 맞춰서 수정, 기본키를 itemId, itemName, itemEffectId로 수정 (개체 무결성)
</commit_message>
<xml_diff>
--- a/Assets/Project/Csv/Item/AdditionalTable/ItemEffectTable.xlsx
+++ b/Assets/Project/Csv/Item/AdditionalTable/ItemEffectTable.xlsx
@@ -5,33 +5,53 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ycjun\OneDrive\문서\Projects\Git\Dairy Farm\Assets\Project\Csv\Item\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ycjun\OneDrive\문서\Projects\Git\Dairy Farm\Assets\Project\Csv\Item\AdditionalTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4692EB7B-BC6C-49C3-B83D-8BF2B584A637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDCD97F-5722-4644-900A-82A7D80BFB63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="enum EffectTriggerType" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>{itemId/int/UNIQUE/NOT NULL}</t>
-  </si>
-  <si>
-    <t>{itemName/string/UNIQUE/NOT NULL}</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>{itemId/int/NOT NULL}</t>
+  </si>
+  <si>
+    <t>{itemName/string/NOT NULL}</t>
+  </si>
+  <si>
+    <t>{itemEffectId/AssetID/NOT NULL}</t>
   </si>
   <si>
     <t>{effectValues/int[]}</t>
   </si>
   <si>
-    <t>{itemEffectId/AssetID/NOT NULL}</t>
+    <t>enum EffectTriggerType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>value</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OnAnimEvent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OnUse</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{triggerType/enum/DEFAULT(OnUse)}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -380,16 +400,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.25" customWidth="1"/>
+    <col min="5" max="5" width="18.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -397,59 +418,109 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E208BEEE-EE79-4E37-B216-C8BB0DE54503}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>